<commit_message>
Compute PR, guarantee tests and the Shapley allocation with res-asset-kpi
The PR family (res_asset_kpi.pv.pr_terms), the contract availability, the
guarantee step-down, tolerance, damages and bonus (res_asset_kpi.pv,
res_asset_kpi.contracts) and the Shapley values of the bridge now come from
res-asset-kpi. The sequential bridge stays here: it applies measured losses to
the model potential in months with almost no production, and the published
tables carry the per-loss energies.

Every value is reproduced to within 2e-16, except one cell: the excluded share
of the night-only 2015 stub period of the PVDAQ systems (local time before the
first UTC day), which has no daylight hours and is now empty instead of 1.0.
</commit_message>
<xml_diff>
--- a/results/pvdaq_1276/report.xlsx
+++ b/results/pvdaq_1276/report.xlsx
@@ -5381,9 +5381,7 @@
       <c r="J2" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K2" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="K2" s="6" t="n"/>
       <c r="L2" s="6" t="n"/>
     </row>
     <row r="3">
@@ -5463,7 +5461,7 @@
         <v>0</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>13.84077970703493</v>
+        <v>13.84077970703494</v>
       </c>
       <c r="K4" s="6" t="n">
         <v>0</v>
@@ -5584,7 +5582,7 @@
         <v>11731.70003581958</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>703.9020021491748</v>
+        <v>703.9020021491747</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>

</xml_diff>